<commit_message>
Preserve current UI source for isolated programming integration
All current source copied and SHA-256 verified; generated artifacts cloned separately. No UI checkout edits.

NOT COVERED: combined release/year verification and device acceptance pending.

Agent: uifixjoin
</commit_message>
<xml_diff>
--- a/docs/EXPOSURE_CONTRACT_REVIEW_2026-07-28.xlsx
+++ b/docs/EXPOSURE_CONTRACT_REVIEW_2026-07-28.xlsx
@@ -3470,12 +3470,12 @@
       </c>
       <c r="I47" s="4" t="inlineStr">
         <is>
-          <t>RULED 2026-07-28</t>
+          <t>RULED 2026-09-07 (R-381)</t>
         </is>
       </c>
       <c r="J47" s="2" t="inlineStr">
         <is>
-          <t>Bible S1: off-season weeks 1-2 are the OPTIONAL block, nothing compulsory.</t>
+          <t>Preparation through week 4: optional light off-feet aerobic offers; no automatic speed. Shared OFFSEASON_PREPARATION policy.</t>
         </is>
       </c>
     </row>
@@ -3522,12 +3522,12 @@
       </c>
       <c r="I48" s="4" t="inlineStr">
         <is>
-          <t>RULED 2026-07-28</t>
+          <t>RULED 2026-09-07 (R-381)</t>
         </is>
       </c>
       <c r="J48" s="2" t="inlineStr">
         <is>
-          <t>Bible S1: off-season weeks 1-2 are the OPTIONAL block, nothing compulsory.</t>
+          <t>Preparation through week 4: optional light off-feet aerobic offers; no automatic speed. Shared OFFSEASON_PREPARATION policy.</t>
         </is>
       </c>
     </row>
@@ -3574,12 +3574,12 @@
       </c>
       <c r="I49" s="4" t="inlineStr">
         <is>
-          <t>RULED 2026-07-28</t>
+          <t>RULED 2026-09-07 (R-381)</t>
         </is>
       </c>
       <c r="J49" s="2" t="inlineStr">
         <is>
-          <t>Bible S1: off-season weeks 1-2 are the OPTIONAL block, nothing compulsory.</t>
+          <t>Preparation through week 4: optional light off-feet aerobic offers; no automatic speed. Shared OFFSEASON_PREPARATION policy.</t>
         </is>
       </c>
     </row>
@@ -4178,7 +4178,7 @@
       </c>
       <c r="E61" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F61" s="5" t="inlineStr">
@@ -4198,12 +4198,12 @@
       </c>
       <c r="I61" s="4" t="inlineStr">
         <is>
-          <t>RULED 2026-07-28</t>
+          <t>RULED 2026-09-07 (R-381)</t>
         </is>
       </c>
       <c r="J61" s="2" t="inlineStr">
         <is>
-          <t>RULED: conditioning counts TOTAL, team training and games included. Weekly cap 5 TOTAL, in-season target 3, max 4 RUNNING sessions year-round, a 5th must be off-legs. S2 amended to state the basis and S3 annotated so its "extra" figures no longer read as a separate budget.</t>
+          <t>Preparation through week 4: optional light off-feet aerobic offers; no automatic speed. Shared OFFSEASON_PREPARATION policy.</t>
         </is>
       </c>
     </row>
@@ -4230,7 +4230,7 @@
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F62" s="5" t="inlineStr">
@@ -4250,12 +4250,12 @@
       </c>
       <c r="I62" s="4" t="inlineStr">
         <is>
-          <t>RULED 2026-07-28</t>
+          <t>RULED 2026-09-07 (R-381)</t>
         </is>
       </c>
       <c r="J62" s="2" t="inlineStr">
         <is>
-          <t>RULED: conditioning counts TOTAL, team training and games included. Weekly cap 5 TOTAL, in-season target 3, max 4 RUNNING sessions year-round, a 5th must be off-legs. S2 amended to state the basis and S3 annotated so its "extra" figures no longer read as a separate budget.</t>
+          <t>Preparation through week 4: optional light off-feet aerobic offers; no automatic speed. Shared OFFSEASON_PREPARATION policy.</t>
         </is>
       </c>
     </row>
@@ -4282,7 +4282,7 @@
       </c>
       <c r="E63" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F63" s="5" t="inlineStr">
@@ -4302,12 +4302,12 @@
       </c>
       <c r="I63" s="4" t="inlineStr">
         <is>
-          <t>RULED 2026-07-28</t>
+          <t>RULED 2026-09-07 (R-381)</t>
         </is>
       </c>
       <c r="J63" s="2" t="inlineStr">
         <is>
-          <t>RULED: conditioning counts TOTAL, team training and games included. Weekly cap 5 TOTAL, in-season target 3, max 4 RUNNING sessions year-round, a 5th must be off-legs. S2 amended to state the basis and S3 annotated so its "extra" figures no longer read as a separate budget.</t>
+          <t>Preparation through week 4: optional light off-feet aerobic offers; no automatic speed. Shared OFFSEASON_PREPARATION policy.</t>
         </is>
       </c>
     </row>
@@ -4334,7 +4334,7 @@
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F64" s="5" t="inlineStr">
@@ -4354,12 +4354,12 @@
       </c>
       <c r="I64" s="4" t="inlineStr">
         <is>
-          <t>RULED 2026-07-28</t>
+          <t>RULED 2026-09-07 (R-381)</t>
         </is>
       </c>
       <c r="J64" s="2" t="inlineStr">
         <is>
-          <t>Bible S2 floor is 1; 2-3 is the usual maximum.</t>
+          <t>Preparation through week 4: optional light off-feet aerobic offers; no automatic speed. Shared OFFSEASON_PREPARATION policy.</t>
         </is>
       </c>
     </row>
@@ -4386,7 +4386,7 @@
       </c>
       <c r="E65" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F65" s="5" t="inlineStr">
@@ -4406,12 +4406,12 @@
       </c>
       <c r="I65" s="4" t="inlineStr">
         <is>
-          <t>RULED 2026-07-28</t>
+          <t>RULED 2026-09-07 (R-381)</t>
         </is>
       </c>
       <c r="J65" s="2" t="inlineStr">
         <is>
-          <t>Bible S2 floor is 1; 2-3 is the usual maximum.</t>
+          <t>Preparation through week 4: optional light off-feet aerobic offers; no automatic speed. Shared OFFSEASON_PREPARATION policy.</t>
         </is>
       </c>
     </row>
@@ -4438,7 +4438,7 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>0</t>
         </is>
       </c>
       <c r="F66" s="5" t="inlineStr">
@@ -4458,12 +4458,12 @@
       </c>
       <c r="I66" s="4" t="inlineStr">
         <is>
-          <t>RULED 2026-07-28</t>
+          <t>RULED 2026-09-07 (R-381)</t>
         </is>
       </c>
       <c r="J66" s="2" t="inlineStr">
         <is>
-          <t>Bible S2 floor is 1; 2-3 is the usual maximum.</t>
+          <t>Preparation through week 4: optional light off-feet aerobic offers; no automatic speed. Shared OFFSEASON_PREPARATION policy.</t>
         </is>
       </c>
     </row>

</xml_diff>